<commit_message>
updated data for 5-6 Days
</commit_message>
<xml_diff>
--- a/12602788.xlsx
+++ b/12602788.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="52">
   <si>
     <t>My Data, My Code — Daily Log</t>
   </si>
@@ -160,6 +160,21 @@
   </si>
   <si>
     <t>Rest day, worked on a Project.</t>
+  </si>
+  <si>
+    <t>Studied DSA and solved Problems.</t>
+  </si>
+  <si>
+    <t>Studied DSA and solved Problems on LeetCode.</t>
+  </si>
+  <si>
+    <t>Travelled out of Station,Studied DSA.</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Studied DSA and solved Problems on LeetCode and c++ on HackerRank.</t>
   </si>
 </sst>
 </file>
@@ -333,7 +348,73 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3174,84 +3255,234 @@
       </c>
     </row>
     <row r="59" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="9"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-      <c r="K59" s="6"/>
-      <c r="L59" s="6"/>
-      <c r="M59" s="6"/>
-      <c r="N59" s="7"/>
+      <c r="A59" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B59" s="4">
+        <v>500</v>
+      </c>
+      <c r="C59" s="4">
+        <v>85</v>
+      </c>
+      <c r="D59" s="4">
+        <v>50</v>
+      </c>
+      <c r="E59" s="4">
+        <v>80</v>
+      </c>
+      <c r="F59" s="4">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4">
+        <v>0</v>
+      </c>
+      <c r="H59" s="4">
+        <v>350</v>
+      </c>
+      <c r="I59" s="5">
+        <f t="shared" ref="I59:I63" si="4">IF(SUM(B59:F59,H59)=0,"",SUM(B59:F59,H59))</f>
+        <v>1065</v>
+      </c>
+      <c r="J59" s="5">
+        <f t="shared" ref="J59:J63" si="5">IF(I59="","",1440-I59)</f>
+        <v>375</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L59" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M59" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="N59" s="7" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="60" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="9"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="6"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="6"/>
-      <c r="N60" s="7"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="3"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
-      <c r="K61" s="6"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="6"/>
-      <c r="N61" s="7"/>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="3"/>
-      <c r="B62" s="4"/>
-      <c r="C62" s="4"/>
-      <c r="D62" s="4"/>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="6"/>
-      <c r="L62" s="6"/>
-      <c r="M62" s="6"/>
-      <c r="N62" s="7"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="3"/>
-      <c r="B63" s="4"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="6"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="6"/>
-      <c r="N63" s="7"/>
+      <c r="A60" s="9">
+        <v>46295</v>
+      </c>
+      <c r="B60" s="4">
+        <v>480</v>
+      </c>
+      <c r="C60" s="4">
+        <v>90</v>
+      </c>
+      <c r="D60" s="4">
+        <v>40</v>
+      </c>
+      <c r="E60" s="4">
+        <v>80</v>
+      </c>
+      <c r="F60" s="4">
+        <v>0</v>
+      </c>
+      <c r="G60" s="4">
+        <v>0</v>
+      </c>
+      <c r="H60" s="4">
+        <v>420</v>
+      </c>
+      <c r="I60" s="5">
+        <f t="shared" si="4"/>
+        <v>1110</v>
+      </c>
+      <c r="J60" s="5">
+        <f t="shared" si="5"/>
+        <v>330</v>
+      </c>
+      <c r="K60" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L60" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M60" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N60" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="9">
+        <v>46296</v>
+      </c>
+      <c r="B61" s="4">
+        <v>410</v>
+      </c>
+      <c r="C61" s="4">
+        <v>0</v>
+      </c>
+      <c r="D61" s="4">
+        <v>60</v>
+      </c>
+      <c r="E61" s="4">
+        <v>60</v>
+      </c>
+      <c r="F61" s="4">
+        <v>0</v>
+      </c>
+      <c r="G61" s="4">
+        <v>0</v>
+      </c>
+      <c r="H61" s="4">
+        <v>480</v>
+      </c>
+      <c r="I61" s="5">
+        <f t="shared" si="4"/>
+        <v>1010</v>
+      </c>
+      <c r="J61" s="5">
+        <f t="shared" si="5"/>
+        <v>430</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L61" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M61" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="N61" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A62" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B62" s="4">
+        <v>430</v>
+      </c>
+      <c r="C62" s="4">
+        <v>0</v>
+      </c>
+      <c r="D62" s="4">
+        <v>60</v>
+      </c>
+      <c r="E62" s="4">
+        <v>80</v>
+      </c>
+      <c r="F62" s="4">
+        <v>0</v>
+      </c>
+      <c r="G62" s="4">
+        <v>0</v>
+      </c>
+      <c r="H62" s="4">
+        <v>420</v>
+      </c>
+      <c r="I62" s="5">
+        <f t="shared" si="4"/>
+        <v>990</v>
+      </c>
+      <c r="J62" s="5">
+        <f t="shared" si="5"/>
+        <v>450</v>
+      </c>
+      <c r="K62" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="L62" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M62" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="N62" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="9">
+        <v>46298</v>
+      </c>
+      <c r="B63" s="4">
+        <v>440</v>
+      </c>
+      <c r="C63" s="4">
+        <v>0</v>
+      </c>
+      <c r="D63" s="4">
+        <v>60</v>
+      </c>
+      <c r="E63" s="4">
+        <v>60</v>
+      </c>
+      <c r="F63" s="4">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4">
+        <v>0</v>
+      </c>
+      <c r="H63" s="4">
+        <v>500</v>
+      </c>
+      <c r="I63" s="5">
+        <f t="shared" si="4"/>
+        <v>1060</v>
+      </c>
+      <c r="J63" s="5">
+        <f t="shared" si="5"/>
+        <v>380</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L63" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N63" s="7" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="3"/>
@@ -8670,8 +8901,33 @@
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J7:J401">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+  <conditionalFormatting sqref="J7:J58 J64:J401">
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J59">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J60">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J61">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J62">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J63">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>